<commit_message>
Updated Output Variables and the negative test validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000952/negative/01/data/unit-test-coreid-FB3407-negative.xlsx
+++ b/rules/CORE-000952/negative/01/data/unit-test-coreid-FB3407-negative.xlsx
@@ -40,7 +40,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -57,12 +57,11 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <color rgb="FF000000"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
+      <color rgb="FF000000"/>
     </font>
     <font>
       <sz val="11"/>
@@ -74,17 +73,8 @@
       <name val="Calibri"/>
       <color rgb="FF000000"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <color rgb="FF000000"/>
-    </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -98,18 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -139,17 +117,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,18 +468,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>3-4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v/>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -527,42 +503,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Adverse Events</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="str">
+      <c r="A4" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>Concomitant/Prior Medications</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>Subject Elements</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>Subject Visits</v>
       </c>
     </row>
@@ -598,162 +574,162 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>AEENDTC</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>2022-01-30</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
-        <v>DM.RFPENDTC</v>
-      </c>
-      <c r="F3" s="2" t="str">
+      <c r="E3" s="4" t="str">
+        <v>RFPENDTC</v>
+      </c>
+      <c r="F3" s="4" t="str">
         <v>2022-01-19</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>11</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>AEENDTC</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F4" s="4" t="str">
         <v>2018-06-14</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="str">
-        <v>DM.RFPENDTC</v>
-      </c>
-      <c r="F5" s="2" t="str">
+      <c r="E5" s="4" t="str">
+        <v>RFPENDTC</v>
+      </c>
+      <c r="F5" s="4" t="str">
         <v>2006-03-19</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
+      <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>cm.xpt</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="4">
         <v>7</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>CMENDTC</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>2022-01-25</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2">
+      <c r="A7" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="4">
         <v>5</v>
       </c>
-      <c r="E7" s="2" t="str">
-        <v>DM.RFPENDTC</v>
-      </c>
-      <c r="F7" s="2" t="str">
+      <c r="E7" s="4" t="str">
+        <v>RFPENDTC</v>
+      </c>
+      <c r="F7" s="4" t="str">
         <v>2022-01-19</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
+      <c r="A8" s="4">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="str">
+      <c r="B8" s="4" t="str">
         <v>se.xpt</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="4">
         <v>7</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E8" s="4" t="str">
         <v>SEENDTC</v>
       </c>
-      <c r="F8" s="2" t="str">
+      <c r="F8" s="4" t="str">
         <v>2022-01-22</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
+      <c r="A9" s="4">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="str">
+      <c r="B9" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C9" s="2" t="str">
+      <c r="C9" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="4">
         <v>5</v>
       </c>
-      <c r="E9" s="2" t="str">
-        <v>DM.RFPENDTC</v>
-      </c>
-      <c r="F9" s="2" t="str">
+      <c r="E9" s="4" t="str">
+        <v>RFPENDTC</v>
+      </c>
+      <c r="F9" s="4" t="str">
         <v>2022-01-19</v>
       </c>
     </row>
@@ -849,55 +825,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Sex</v>
       </c>
       <c r="R2" s="6" t="str">
@@ -1089,322 +1065,322 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>100001</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>2018-02-20T09:40</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>2019-02-20T10:38</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-01-24</v>
       </c>
       <c r="J5" s="7" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="K5" s="2" t="str">
+      <c r="K5" s="4" t="str">
         <v/>
       </c>
-      <c r="L5" s="4" t="str">
+      <c r="L5" s="5" t="str">
         <v/>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="5">
         <v>360001</v>
       </c>
-      <c r="N5" s="4" t="str">
+      <c r="N5" s="5" t="str">
         <v>1954-08-06</v>
       </c>
-      <c r="O5" s="4" t="str">
+      <c r="O5" s="5" t="str">
         <v>63</v>
       </c>
-      <c r="P5" s="4" t="str">
+      <c r="P5" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="4" t="str">
+      <c r="Q5" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="4" t="str">
+      <c r="R5" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="4" t="str">
+      <c r="S5" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="4" t="str">
+      <c r="T5" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U5" s="4" t="str">
+      <c r="U5" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V5" s="4" t="str">
+      <c r="V5" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W5" s="4" t="str">
+      <c r="W5" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X5" s="4" t="str">
+      <c r="X5" s="5" t="str">
         <v/>
       </c>
-      <c r="Y5" s="4" t="str">
+      <c r="Y5" s="5" t="str">
         <v/>
       </c>
-      <c r="Z5" s="4" t="str">
+      <c r="Z5" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="5" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>100002</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>2018-04-17T09:25</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>2019-03-13</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="5" t="str">
         <v>2018-04-17T09:25</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>2019-03-13</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-03-22</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2019-09-29</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="5" t="str">
         <v>2019-09-29</v>
       </c>
-      <c r="L6" s="4" t="str">
+      <c r="L6" s="5" t="str">
         <v>Y</v>
       </c>
-      <c r="M6" s="4">
+      <c r="M6" s="5">
         <v>360001</v>
       </c>
-      <c r="N6" s="4" t="str">
+      <c r="N6" s="5" t="str">
         <v>1941-07-03</v>
       </c>
-      <c r="O6" s="4" t="str">
+      <c r="O6" s="5" t="str">
         <v>76</v>
       </c>
-      <c r="P6" s="4" t="str">
+      <c r="P6" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q6" s="4" t="str">
+      <c r="Q6" s="5" t="str">
         <v>F</v>
       </c>
-      <c r="R6" s="4" t="str">
+      <c r="R6" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S6" s="4" t="str">
+      <c r="S6" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="4" t="str">
+      <c r="T6" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U6" s="4" t="str">
+      <c r="U6" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V6" s="4" t="str">
+      <c r="V6" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W6" s="4" t="str">
+      <c r="W6" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X6" s="4" t="str">
+      <c r="X6" s="5" t="str">
         <v/>
       </c>
-      <c r="Y6" s="4" t="str">
+      <c r="Y6" s="5" t="str">
         <v/>
       </c>
-      <c r="Z6" s="4" t="str">
+      <c r="Z6" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="5" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>100003</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>2018-04-18T09:30</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>2018-07-18T11:15</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>2018-04-18T09:30</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>2018-07-18T11:15</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2018-03-22</v>
       </c>
       <c r="J7" s="7" t="str">
         <v>2006-03-19</v>
       </c>
-      <c r="K7" s="2" t="str">
+      <c r="K7" s="4" t="str">
         <v/>
       </c>
-      <c r="L7" s="2" t="str">
+      <c r="L7" s="4" t="str">
         <v/>
       </c>
-      <c r="M7" s="4">
+      <c r="M7" s="5">
         <v>360001</v>
       </c>
-      <c r="N7" s="4" t="str">
+      <c r="N7" s="5" t="str">
         <v>1964-10-28</v>
       </c>
-      <c r="O7" s="4" t="str">
+      <c r="O7" s="5" t="str">
         <v>53</v>
       </c>
-      <c r="P7" s="4" t="str">
+      <c r="P7" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q7" s="4" t="str">
+      <c r="Q7" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R7" s="4" t="str">
+      <c r="R7" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S7" s="4" t="str">
+      <c r="S7" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="4" t="str">
+      <c r="T7" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="U7" s="4" t="str">
+      <c r="U7" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="V7" s="4" t="str">
+      <c r="V7" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="W7" s="4" t="str">
+      <c r="W7" s="5" t="str">
         <v>Drug Ikd</v>
       </c>
-      <c r="X7" s="4" t="str">
+      <c r="X7" s="5" t="str">
         <v/>
       </c>
-      <c r="Y7" s="4" t="str">
+      <c r="Y7" s="5" t="str">
         <v/>
       </c>
-      <c r="Z7" s="4" t="str">
+      <c r="Z7" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="str">
+      <c r="A8" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="5" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="5" t="str">
         <v>CDISC004</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="5">
         <v>200004</v>
       </c>
-      <c r="E8" s="4" t="str">
+      <c r="E8" s="5" t="str">
         <v/>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="5" t="str">
         <v/>
       </c>
-      <c r="G8" s="4" t="str">
+      <c r="G8" s="5" t="str">
         <v/>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="5" t="str">
         <v/>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="5" t="str">
         <v>2018-04-16</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="5" t="str">
         <v>2018-05-04</v>
       </c>
-      <c r="K8" s="2" t="str">
+      <c r="K8" s="4" t="str">
         <v/>
       </c>
-      <c r="L8" s="2" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="5">
         <v>360002</v>
       </c>
-      <c r="N8" s="4" t="str">
+      <c r="N8" s="5" t="str">
         <v>1940-08-14</v>
       </c>
-      <c r="O8" s="4" t="str">
+      <c r="O8" s="5" t="str">
         <v>77</v>
       </c>
-      <c r="P8" s="4" t="str">
+      <c r="P8" s="5" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q8" s="4" t="str">
+      <c r="Q8" s="5" t="str">
         <v>M</v>
       </c>
-      <c r="R8" s="4" t="str">
+      <c r="R8" s="5" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S8" s="4" t="str">
+      <c r="S8" s="5" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T8" s="4" t="str">
+      <c r="T8" s="5" t="str">
         <v/>
       </c>
-      <c r="U8" s="4" t="str">
+      <c r="U8" s="5" t="str">
         <v/>
       </c>
-      <c r="V8" s="4" t="str">
+      <c r="V8" s="5" t="str">
         <v/>
       </c>
-      <c r="W8" s="4" t="str">
+      <c r="W8" s="5" t="str">
         <v/>
       </c>
-      <c r="X8" s="4" t="str">
+      <c r="X8" s="5" t="str">
         <v>Screen Failure</v>
       </c>
-      <c r="Y8" s="4" t="str">
+      <c r="Y8" s="5" t="str">
         <v/>
       </c>
-      <c r="Z8" s="4" t="str">
+      <c r="Z8" s="5" t="str">
         <v>AUS</v>
       </c>
     </row>
@@ -1548,226 +1524,226 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="8" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="5" t="str">
         <v>INFUSION ASSOCIATE REACTION</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>1</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="4" t="str">
+      <c r="D6" s="5" t="str">
         <v>INSOMNIA</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="5" t="str">
         <v>2018-02-22</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>3</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-10-30</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>253</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C7" s="8" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="4" t="str">
+      <c r="D7" s="5" t="str">
         <v>LETHARGY</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>2018-02-22</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>3</v>
       </c>
       <c r="I7" s="7" t="str">
         <v>2022-01-30</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="5" t="str">
         <v>113</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="4" t="str">
+      <c r="B8" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="4" t="str">
+      <c r="D8" s="5" t="str">
         <v>LEFT HIP PAIN CAUSE UNKNOWN</v>
       </c>
-      <c r="E8" s="4" t="str">
+      <c r="E8" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G8" s="4" t="str">
+      <c r="G8" s="5" t="str">
         <v>2018-04-16</v>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="5" t="str">
         <v>2018-04-23</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="5" t="str">
         <v>7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="str">
+      <c r="A9" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B9" s="4" t="str">
+      <c r="B9" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C9" s="8" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D9" s="4" t="str">
+      <c r="D9" s="5" t="str">
         <v>FATIGUE</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G9" s="4" t="str">
+      <c r="G9" s="5" t="str">
         <v>2018-05-02</v>
       </c>
-      <c r="H9" s="4" t="str">
+      <c r="H9" s="5" t="str">
         <v>16</v>
       </c>
-      <c r="I9" s="4" t="str">
+      <c r="I9" s="5" t="str">
         <v>2019-03</v>
       </c>
-      <c r="J9" s="4" t="str">
+      <c r="J9" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="str">
+      <c r="A10" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B10" s="4" t="str">
+      <c r="B10" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D10" s="4" t="str">
+      <c r="D10" s="5" t="str">
         <v>CALF PAIN</v>
       </c>
-      <c r="E10" s="4" t="str">
+      <c r="E10" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F10" s="4" t="str">
+      <c r="F10" s="5" t="str">
         <v>NOT RECOVERED/NOT RESOLVED</v>
       </c>
-      <c r="G10" s="4" t="str">
+      <c r="G10" s="5" t="str">
         <v>2018-07-10</v>
       </c>
-      <c r="H10" s="4" t="str">
+      <c r="H10" s="5" t="str">
         <v>84</v>
       </c>
-      <c r="I10" s="4" t="str">
+      <c r="I10" s="5" t="str">
         <v/>
       </c>
-      <c r="J10" s="4" t="str">
+      <c r="J10" s="5" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="4" t="str">
+      <c r="B11" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC003</v>
       </c>
-      <c r="D11" s="4" t="str">
+      <c r="D11" s="5" t="str">
         <v>DELIRIUM</v>
       </c>
-      <c r="E11" s="4" t="str">
+      <c r="E11" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="F11" s="4" t="str">
+      <c r="F11" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="G11" s="4" t="str">
+      <c r="G11" s="5" t="str">
         <v>2018-05-18</v>
       </c>
-      <c r="H11" s="4" t="str">
+      <c r="H11" s="5" t="str">
         <v>2</v>
       </c>
       <c r="I11" s="7" t="str">
         <v>2018-06-14</v>
       </c>
-      <c r="J11" s="4" t="str">
+      <c r="J11" s="5" t="str">
         <v>29</v>
       </c>
     </row>
@@ -1923,102 +1899,102 @@
       </c>
     </row>
     <row r="5" xml:space="preserve">
-      <c r="A5" s="8" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>CM</v>
       </c>
-      <c r="C5" s="8" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="8" t="str">
+      <c r="D5" s="4" t="str">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>VALACICLOVIR 500 MG</v>
       </c>
-      <c r="F5" s="4" t="str" xml:space="preserve">
+      <c r="F5" s="5" t="str" xml:space="preserve">
         <v xml:space="preserve">CMDECOD
 VALACICLOVIR</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="4" t="str">
         <v>MEDICATION</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>CM</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="8" t="str">
+      <c r="D6" s="4" t="str">
         <v>2</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>G-CSF 480 MCG</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>CMDECOD GRANULOCYTE COLONY STIMULATING FACTOR</v>
       </c>
-      <c r="G6" s="2" t="str">
+      <c r="G6" s="4" t="str">
         <v>MEDICATION</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>2018-02-27</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="4">
         <v>8</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2018-03-03</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="4">
         <v>12</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>CM</v>
       </c>
-      <c r="C7" s="8" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="8" t="str">
+      <c r="D7" s="4" t="str">
         <v>3</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>TYELENOL 5 ml</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>XXXX</v>
       </c>
-      <c r="G7" s="2" t="str">
+      <c r="G7" s="4" t="str">
         <v>MEDICATION</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>2022-01-19</v>
       </c>
-      <c r="I7" s="2">
+      <c r="I7" s="4">
         <v>400</v>
       </c>
-      <c r="J7" s="9" t="str">
+      <c r="J7" s="7" t="str">
         <v>2022-01-25</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="4">
         <v>406</v>
       </c>
     </row>
@@ -2186,116 +2162,116 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>SE</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>SCRN</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>Screen</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="5">
         <v>1</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-01-24</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>2006-03-10</v>
       </c>
-      <c r="K5" s="4" t="str">
+      <c r="K5" s="5" t="str">
         <v>-27</v>
       </c>
-      <c r="L5" s="4" t="str">
+      <c r="L5" s="5" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>SE</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>IKD</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>Treatment IKD</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <v>2</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-12-20T09:40</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2019-03-22T10:38</v>
       </c>
-      <c r="K6" s="4" t="str">
+      <c r="K6" s="5" t="str">
         <v>1</v>
       </c>
-      <c r="L6" s="4" t="str">
+      <c r="L6" s="5" t="str">
         <v>396</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>SE</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>3</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>FU</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>Follow-up</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="5">
         <v>3</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>FOLLOW-UP</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2019-03-22T10:38</v>
       </c>
       <c r="J7" s="7" t="str">
         <v>2022-01-22</v>
       </c>
-      <c r="K7" s="4" t="str">
+      <c r="K7" s="5" t="str">
         <v>396</v>
       </c>
-      <c r="L7" s="4" t="str">
+      <c r="L7" s="5" t="str">
         <v>1430</v>
       </c>
     </row>
@@ -2439,98 +2415,98 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="str">
+      <c r="A5" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B5" s="4" t="str">
+      <c r="B5" s="5" t="str">
         <v>SV</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="4" t="str">
+      <c r="D5" s="5" t="str">
         <v>0</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>-21</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v>2018-01-24</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="str">
+      <c r="A6" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="4" t="str">
+      <c r="B6" s="5" t="str">
         <v>SV</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="4" t="str">
+      <c r="D6" s="5" t="str">
         <v>110</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>CYCLE 1 DAY 1</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>1</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="5" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v>2018-02-15T17:38</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-02-20T16:31:00</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="str">
+      <c r="A7" s="5" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B7" s="4" t="str">
+      <c r="B7" s="5" t="str">
         <v>SV</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="5" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="4" t="str">
+      <c r="D7" s="5" t="str">
         <v>120</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>CYCLE 1 DAY 2</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>2</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="H7" s="4" t="str">
+      <c r="H7" s="5" t="str">
         <v>2018-02-21</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2018-02-21T12:05</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="5" t="str">
         <v>2</v>
       </c>
     </row>

</xml_diff>